<commit_message>
Improve dashboard chart and final portfolio presentation
</commit_message>
<xml_diff>
--- a/output/master_report.xlsx
+++ b/output/master_report.xlsx
@@ -322,165 +322,31 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Data Quality Issues by Worksheet</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Dashboard'!C12</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Dashboard'!$A$13:$A$15</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Dashboard'!$C$13:$C$15</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Dashboard'!D12</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Dashboard'!$A$13:$A$15</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Dashboard'!$D$13:$D$15</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t/>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Issues</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="b"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>19</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7920000" cy="3600000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
+    <ext cx="10001250" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
     <clientData/>
   </oneCellAnchor>
 </wsDr>

</xml_diff>